<commit_message>
Updated engine usage file with correct data
</commit_message>
<xml_diff>
--- a/ZZ383 Engine Usage.xlsx
+++ b/ZZ383 Engine Usage.xlsx
@@ -2033,6 +2033,726 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>WC/PMP/6220011/50/A</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>WILDCAT OVERSPEED 115% TO 118% NR</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LK2113</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>WG1369-2370-041</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>WC/PMP/6220011/50/A</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>WILDCAT OVERSPEED 115% TO 118% NR</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LK2114</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>WG1369-2370-041</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>45.00</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>50.00</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>WC/OVERSPEED/10/A</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>WILDCAT OVERSPEED 118% TO 120% NR</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>WILDCAT</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>20000.00</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>20000.00</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>19999.00</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>WC/PMP/6220011/10/A</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>WILDCAT OVERSPEED 118% TO 120% NR</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LK2109</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>WG1369-2370-041</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>WC/PMP/6220011/10/A</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>WILDCAT OVERSPEED 118% TO 120% NR</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LK2111</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>WG1369-2370-041</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>WC/PMP/6220011/10/A</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>WILDCAT OVERSPEED 118% TO 120% NR</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LK2113</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>WG1369-2370-041</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>WC/PMP/6220011/10/A</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>WILDCAT OVERSPEED 118% TO 120% NR</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LK2114</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>WG1369-2370-041</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>8.00</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RL</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>WC/RUN/LANDINGS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>RUNNING LANDINGS MASTER LIFE</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>WILDCAT</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>99999.00</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>99999.00</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>99216.00</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>783.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>WCRSSC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ROTOR START/STOP CYCLES</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>ROTOR START/STOP CYCLES</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>WILDCAT</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>20000.00</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>20000.00</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>18502.00</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>1498.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>XJ</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>WC/GRD/TAXI</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>GROUND TAXI MASTER LIFE</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>WILDCAT</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>K0058</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>20000:00</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>20000:00</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>19888:36</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>0:00</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>111:24</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated file including SM / SN interval types
</commit_message>
<xml_diff>
--- a/ZZ383 Engine Usage.xlsx
+++ b/ZZ383 Engine Usage.xlsx
@@ -2684,70 +2684,214 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>SM</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>WC/STARTS/ECU</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>T800 ENGINE STARTS</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>P4N155</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>LH70120-01</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>64643</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>8866.00</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>1134.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>SN</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>WC/STARTS/ECU</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>T800 ENGINE STARTS</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>P4N175</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>LH70120-01</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>64643</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>10000.0</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>8537.00</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>1463.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>XJ</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>WC/GRD/TAXI</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>GROUND TAXI MASTER LIFE</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>ZZ383</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>WILDCAT</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>K0058</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>20000:00</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="J38" t="inlineStr">
         <is>
           <t>20000:00</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>ZZ383</t>
-        </is>
-      </c>
-      <c r="L36" t="inlineStr">
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ZZ383</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
         <is>
           <t>19888:36</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M38" t="inlineStr">
         <is>
           <t>0:00</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>111:24</t>
         </is>

</xml_diff>